<commit_message>
Demo: fechas relativas a hoy y ejemplos del formulario de distintos campos
- La demo guarda su fecha de construcción (DEMO_FECHA) y app.js mueve todas las
  fechas (seguimientos, historial, cartas) a partir de hoy al cargar la página.
- Ejemplos del perfil variados: Analista de datos, Contador, Diseñador UX,
  Supervisor de logística; Excel, contabilidad, Figma, atención al cliente.
- Instrucciones de GitHub Pages con la rama main.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/oportunidades-demo.xlsx
+++ b/docs/oportunidades-demo.xlsx
@@ -662,7 +662,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20T11:00:04</t>
+          <t>2026-10-20T11:26:55</t>
         </is>
       </c>
     </row>
@@ -1907,7 +1907,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 11:00:04</t>
+          <t>2026-10-20 11:26:55</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -1930,7 +1930,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 11:00:04</t>
+          <t>2026-10-20 11:26:55</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -1953,7 +1953,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 11:00:04</t>
+          <t>2026-10-20 11:26:55</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -1976,7 +1976,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 11:00:04</t>
+          <t>2026-10-20 11:26:55</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -1999,7 +1999,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 11:00:04</t>
+          <t>2026-10-20 11:26:55</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -2022,7 +2022,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 11:00:04</t>
+          <t>2026-10-20 11:26:55</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -2045,7 +2045,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 11:00:04</t>
+          <t>2026-10-20 11:26:55</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -2068,7 +2068,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 11:00:04</t>
+          <t>2026-10-20 11:26:55</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -2091,7 +2091,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 11:00:04</t>
+          <t>2026-10-20 11:26:55</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -2114,7 +2114,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 11:00:04</t>
+          <t>2026-10-20 11:26:55</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -2137,7 +2137,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 11:00:04</t>
+          <t>2026-10-20 11:26:55</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -2160,7 +2160,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 11:00:04</t>
+          <t>2026-10-20 11:26:55</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -2183,7 +2183,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 11:00:04</t>
+          <t>2026-10-20 11:26:55</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -2206,7 +2206,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 11:00:04</t>
+          <t>2026-10-20 11:26:55</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -2229,7 +2229,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 11:00:04</t>
+          <t>2026-10-20 11:26:55</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -2252,7 +2252,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 11:00:04</t>
+          <t>2026-10-20 11:26:55</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Buscador de habilidades al estilo LinkedIn: nombres cortos en vez de frases de ESCO
- Lista nueva (2.594): conocimientos de ESCO de hasta 4 palabras, competencias
  de ESCO muy usadas reescritas como nombre corto (con su URI) y herramientas y
  métodos curados que ESCO no tiene (marcados «curada»).
- Buscador desde 2 letras, solo al inicio de palabra: exacta, empieza por, una
  palabra empieza por; dentro de cada grupo, la más usada primero.
- Inglés debajo solo si es distinto. Atribución actualizada (versión adaptada).
- Índice: 0,98 MB (0,21 MB con gzip), antes 2,73 MB.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/oportunidades-demo.xlsx
+++ b/docs/oportunidades-demo.xlsx
@@ -662,7 +662,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20T12:47:46</t>
+          <t>2026-10-20T15:40:48</t>
         </is>
       </c>
     </row>
@@ -1907,7 +1907,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 12:47:46</t>
+          <t>2026-10-20 15:40:48</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -1930,7 +1930,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 12:47:46</t>
+          <t>2026-10-20 15:40:48</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -1953,7 +1953,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 12:47:46</t>
+          <t>2026-10-20 15:40:48</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -1976,7 +1976,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 12:47:46</t>
+          <t>2026-10-20 15:40:48</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -1999,7 +1999,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 12:47:46</t>
+          <t>2026-10-20 15:40:48</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -2022,7 +2022,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 12:47:46</t>
+          <t>2026-10-20 15:40:48</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -2045,7 +2045,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 12:47:46</t>
+          <t>2026-10-20 15:40:48</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -2068,7 +2068,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 12:47:46</t>
+          <t>2026-10-20 15:40:48</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -2091,7 +2091,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 12:47:46</t>
+          <t>2026-10-20 15:40:48</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -2114,7 +2114,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 12:47:46</t>
+          <t>2026-10-20 15:40:48</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -2137,7 +2137,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 12:47:46</t>
+          <t>2026-10-20 15:40:48</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -2160,7 +2160,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 12:47:46</t>
+          <t>2026-10-20 15:40:48</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -2183,7 +2183,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 12:47:46</t>
+          <t>2026-10-20 15:40:48</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -2206,7 +2206,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 12:47:46</t>
+          <t>2026-10-20 15:40:48</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -2229,7 +2229,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 12:47:46</t>
+          <t>2026-10-20 15:40:48</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -2252,7 +2252,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 12:47:46</t>
+          <t>2026-10-20 15:40:48</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Habilidades curadas con equivalente en ESCO para sugerir ocupaciones
Las curadas pueden llevar «esco_equivalente» (Excel → hojas de cálculo, Power BI → Business Intelligence,
Salesforce → CRM). Al buscar ocupaciones, tener la curada cuenta como tener esa habilidad de ESCO.
112 curadas enlazadas, solo donde la equivalencia es clara. Se añaden 59 habilidades de ESCO con nombre
corto para que haya a qué apuntar (CRM, Procesadores de texto, Manejo de caja…).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/oportunidades-demo.xlsx
+++ b/docs/oportunidades-demo.xlsx
@@ -662,7 +662,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20T15:40:48</t>
+          <t>2026-10-20T17:08:45</t>
         </is>
       </c>
     </row>
@@ -1907,7 +1907,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 15:40:48</t>
+          <t>2026-10-20 17:08:45</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -1930,7 +1930,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 15:40:48</t>
+          <t>2026-10-20 17:08:45</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -1953,7 +1953,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 15:40:48</t>
+          <t>2026-10-20 17:08:45</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -1976,7 +1976,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 15:40:48</t>
+          <t>2026-10-20 17:08:45</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -1999,7 +1999,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 15:40:48</t>
+          <t>2026-10-20 17:08:45</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -2022,7 +2022,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 15:40:48</t>
+          <t>2026-10-20 17:08:45</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -2045,7 +2045,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 15:40:48</t>
+          <t>2026-10-20 17:08:45</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -2068,7 +2068,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 15:40:48</t>
+          <t>2026-10-20 17:08:45</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -2091,7 +2091,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 15:40:48</t>
+          <t>2026-10-20 17:08:45</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -2114,7 +2114,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 15:40:48</t>
+          <t>2026-10-20 17:08:45</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -2137,7 +2137,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 15:40:48</t>
+          <t>2026-10-20 17:08:45</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -2160,7 +2160,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 15:40:48</t>
+          <t>2026-10-20 17:08:45</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -2183,7 +2183,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 15:40:48</t>
+          <t>2026-10-20 17:08:45</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -2206,7 +2206,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 15:40:48</t>
+          <t>2026-10-20 17:08:45</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -2229,7 +2229,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 15:40:48</t>
+          <t>2026-10-20 17:08:44</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -2252,7 +2252,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 15:40:48</t>
+          <t>2026-10-20 17:08:44</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Nombres de habilidad sin paréntesis: la sigla pasa a sinónimo
«Punto de venta (POS)» → «Punto de venta», con «POS» como sinónimo; igual con EPP, QA, LLM, AML y BIM.
Las siglas de ESCO también van como sinónimo al construir el índice. En el mapa de áreas, las habilidades
con paréntesis pasan a su nombre en la lista («CRM (Salesforce, HubSpot)» → «CRM»); nueva curada
«Sistemas de reservas» (Opera, PMS). Así la razón ya no queda «(por tu Punto de venta (POS))».

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/oportunidades-demo.xlsx
+++ b/docs/oportunidades-demo.xlsx
@@ -662,7 +662,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20T17:08:45</t>
+          <t>2026-10-20T17:20:30</t>
         </is>
       </c>
     </row>
@@ -1907,7 +1907,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:08:45</t>
+          <t>2026-10-20 17:20:30</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -1930,7 +1930,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:08:45</t>
+          <t>2026-10-20 17:20:30</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -1953,7 +1953,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:08:45</t>
+          <t>2026-10-20 17:20:30</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -1976,7 +1976,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:08:45</t>
+          <t>2026-10-20 17:20:30</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -1999,7 +1999,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:08:45</t>
+          <t>2026-10-20 17:20:30</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -2022,7 +2022,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:08:45</t>
+          <t>2026-10-20 17:20:30</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -2045,7 +2045,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:08:45</t>
+          <t>2026-10-20 17:20:30</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -2068,7 +2068,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:08:45</t>
+          <t>2026-10-20 17:20:30</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -2091,7 +2091,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:08:45</t>
+          <t>2026-10-20 17:20:30</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -2114,7 +2114,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:08:45</t>
+          <t>2026-10-20 17:20:30</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -2137,7 +2137,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:08:45</t>
+          <t>2026-10-20 17:20:30</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -2160,7 +2160,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:08:45</t>
+          <t>2026-10-20 17:20:30</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -2183,7 +2183,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:08:45</t>
+          <t>2026-10-20 17:20:30</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -2206,7 +2206,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:08:45</t>
+          <t>2026-10-20 17:20:30</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -2229,7 +2229,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:08:44</t>
+          <t>2026-10-20 17:20:30</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -2252,7 +2252,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:08:44</t>
+          <t>2026-10-20 17:20:30</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Ventana de la app más pequeña
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/oportunidades-demo.xlsx
+++ b/docs/oportunidades-demo.xlsx
@@ -662,7 +662,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20T17:20:30</t>
+          <t>2026-10-21T10:29:28</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>2026-10-23 · Entrevista</t>
+          <t>2026-10-24 · Entrevista</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -693,7 +693,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25 · Contacté</t>
+          <t>2026-10-26 · Contacté</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -705,7 +705,7 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>2026-10-27 · Aplicado</t>
+          <t>2026-10-28 · Aplicado</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -996,7 +996,7 @@
       <c r="Y2" s="3" t="inlineStr"/>
       <c r="Z2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1113,7 +1113,7 @@
       <c r="Y3" s="3" t="inlineStr"/>
       <c r="Z3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1237,7 +1237,7 @@
       </c>
       <c r="Z4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       <c r="V5" s="3" t="inlineStr"/>
       <c r="W5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="X5" s="11" t="inlineStr">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="Z5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1474,7 @@
       <c r="V6" s="3" t="inlineStr"/>
       <c r="W6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="X6" s="11" t="inlineStr">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="Z6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1600,7 @@
       <c r="V7" s="3" t="inlineStr"/>
       <c r="W7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="X7" s="11" t="inlineStr">
@@ -1615,7 +1615,7 @@
       </c>
       <c r="Z7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1764,7 +1764,7 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1805,7 +1805,7 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1846,7 +1846,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1907,7 +1907,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:20:30</t>
+          <t>2026-10-21 10:29:28</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -1930,7 +1930,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:20:30</t>
+          <t>2026-10-21 10:29:28</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -1953,7 +1953,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:20:30</t>
+          <t>2026-10-21 10:29:28</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -1976,7 +1976,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:20:30</t>
+          <t>2026-10-21 10:29:28</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -1999,7 +1999,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:20:30</t>
+          <t>2026-10-21 10:29:28</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -2022,7 +2022,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:20:30</t>
+          <t>2026-10-21 10:29:28</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -2045,7 +2045,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:20:30</t>
+          <t>2026-10-21 10:29:28</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -2068,7 +2068,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:20:30</t>
+          <t>2026-10-21 10:29:28</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -2091,7 +2091,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:20:30</t>
+          <t>2026-10-21 10:29:28</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -2114,7 +2114,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:20:30</t>
+          <t>2026-10-21 10:29:28</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -2137,7 +2137,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:20:30</t>
+          <t>2026-10-21 10:29:28</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -2160,7 +2160,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:20:30</t>
+          <t>2026-10-21 10:29:28</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -2183,7 +2183,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:20:30</t>
+          <t>2026-10-21 10:29:28</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -2206,7 +2206,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:20:30</t>
+          <t>2026-10-21 10:29:28</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -2229,7 +2229,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:20:30</t>
+          <t>2026-10-21 10:29:28</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -2252,7 +2252,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 17:20:30</t>
+          <t>2026-10-21 10:29:28</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Mi perfil como encuesta
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/oportunidades-demo.xlsx
+++ b/docs/oportunidades-demo.xlsx
@@ -662,7 +662,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21T10:29:28</t>
+          <t>2026-10-21T10:48:32</t>
         </is>
       </c>
     </row>
@@ -1907,7 +1907,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:29:28</t>
+          <t>2026-10-21 10:48:32</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -1930,7 +1930,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:29:28</t>
+          <t>2026-10-21 10:48:32</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -1953,7 +1953,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:29:28</t>
+          <t>2026-10-21 10:48:32</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -1976,7 +1976,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:29:28</t>
+          <t>2026-10-21 10:48:32</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -1999,7 +1999,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:29:28</t>
+          <t>2026-10-21 10:48:32</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -2022,7 +2022,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:29:28</t>
+          <t>2026-10-21 10:48:32</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -2045,7 +2045,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:29:28</t>
+          <t>2026-10-21 10:48:32</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -2068,7 +2068,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:29:28</t>
+          <t>2026-10-21 10:48:32</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -2091,7 +2091,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:29:28</t>
+          <t>2026-10-21 10:48:32</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -2114,7 +2114,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:29:28</t>
+          <t>2026-10-21 10:48:32</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -2137,7 +2137,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:29:28</t>
+          <t>2026-10-21 10:48:32</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -2160,7 +2160,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:29:28</t>
+          <t>2026-10-21 10:48:32</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -2183,7 +2183,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:29:28</t>
+          <t>2026-10-21 10:48:32</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -2206,7 +2206,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:29:28</t>
+          <t>2026-10-21 10:48:32</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -2229,7 +2229,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:29:28</t>
+          <t>2026-10-21 10:48:32</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -2252,7 +2252,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:29:28</t>
+          <t>2026-10-21 10:48:32</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Contactos: quién dirige el área, con fuente pública
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EMgAjCZzSZtbDYapbjrcRY
</commit_message>
<xml_diff>
--- a/docs/oportunidades-demo.xlsx
+++ b/docs/oportunidades-demo.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Empresas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Vacantes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Seguimiento" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empresas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vacantes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$1:$B$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Empresas'!$A$1:$Z$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Empresas'!$A$1:$AA$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Vacantes'!$A$1:$I$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Seguimiento'!$A$1:$E$17</definedName>
   </definedNames>
@@ -662,7 +662,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21T10:48:32</t>
+          <t>2026-10-28T14:52:57</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>2026-10-24 · Entrevista</t>
+          <t>2026-10-31 · Entrevista</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -693,7 +693,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>2026-10-26 · Contacté</t>
+          <t>2026-11-02 · Contacté</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -705,7 +705,7 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>2026-10-28 · Aplicado</t>
+          <t>2026-11-04 · Aplicado</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -726,7 +726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z7"/>
+  <dimension ref="A1:AA7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -745,16 +745,17 @@
     <col width="32" customWidth="1" min="14" max="14"/>
     <col width="32" customWidth="1" min="15" max="15"/>
     <col width="32" customWidth="1" min="16" max="16"/>
-    <col width="36" customWidth="1" min="17" max="17"/>
-    <col width="56" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
-    <col width="10" customWidth="1" min="20" max="20"/>
-    <col width="34" customWidth="1" min="21" max="21"/>
-    <col width="30" customWidth="1" min="22" max="22"/>
-    <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="30" customWidth="1" min="24" max="24"/>
+    <col width="44" customWidth="1" min="17" max="17"/>
+    <col width="36" customWidth="1" min="18" max="18"/>
+    <col width="56" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="34" customWidth="1" min="22" max="22"/>
+    <col width="30" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
     <col width="30" customWidth="1" min="25" max="25"/>
-    <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="30" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -840,50 +841,55 @@
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Roles a contactar</t>
+          <t>Personas a contactar</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Búsqueda LinkedIn</t>
+          <t>Cargos a contactar</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
           <t>Vacantes</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Vacantes abiertas</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Nota de rastreo</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Seguimiento</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Mensaje</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Carta</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Descubierta</t>
         </is>
@@ -970,33 +976,34 @@
           <t>https://www.linkedin.com/search/results/companies/?keywords=Banco+Quisqueya+Digital+%28demo%29</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr">
+      <c r="Q2" s="3" t="inlineStr"/>
+      <c r="R2" s="3" t="inlineStr">
         <is>
           <t>Gerente de Innovación; Head of Data</t>
         </is>
       </c>
-      <c r="R2" s="11" t="inlineStr">
+      <c r="S2" s="11" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/search/results/people/?keywords=Gerente+de+Innovaci%C3%B3n+Banco+Quisqueya+Digital+%28demo%29
 https://www.linkedin.com/search/results/people/?keywords=Head+of+Data+Banco+Quisqueya+Digital+%28demo%29</t>
         </is>
       </c>
-      <c r="S2" s="3" t="inlineStr">
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>no hay</t>
         </is>
       </c>
-      <c r="T2" s="3" t="n">
+      <c r="U2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="U2" s="3" t="inlineStr"/>
       <c r="V2" s="3" t="inlineStr"/>
       <c r="W2" s="3" t="inlineStr"/>
       <c r="X2" s="3" t="inlineStr"/>
       <c r="Y2" s="3" t="inlineStr"/>
-      <c r="Z2" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
+      <c r="Z2" s="3" t="inlineStr"/>
+      <c r="AA2" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -1084,36 +1091,37 @@
           <t>https://www.linkedin.com/search/results/companies/?keywords=Nube+Ta%C3%ADna+Labs+%28demo%29</t>
         </is>
       </c>
-      <c r="Q3" s="3" t="inlineStr">
+      <c r="Q3" s="3" t="inlineStr"/>
+      <c r="R3" s="3" t="inlineStr">
         <is>
           <t>Fundador / CTO</t>
         </is>
       </c>
-      <c r="R3" s="12" t="inlineStr">
+      <c r="S3" s="12" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/search/results/people/?keywords=Fundador+%2F+CTO+Nube+Ta%C3%ADna+Labs+%28demo%29</t>
         </is>
       </c>
-      <c r="S3" s="3" t="inlineStr">
+      <c r="T3" s="3" t="inlineStr">
         <is>
           <t>abrir manualmente</t>
         </is>
       </c>
-      <c r="T3" s="3" t="n">
+      <c r="U3" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="U3" s="11" t="inlineStr">
+      <c r="V3" s="11" t="inlineStr">
         <is>
           <t>La página de empleos necesita JavaScript.</t>
         </is>
       </c>
-      <c r="V3" s="3" t="inlineStr"/>
       <c r="W3" s="3" t="inlineStr"/>
       <c r="X3" s="3" t="inlineStr"/>
       <c r="Y3" s="3" t="inlineStr"/>
-      <c r="Z3" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
+      <c r="Z3" s="3" t="inlineStr"/>
+      <c r="AA3" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -1203,41 +1211,42 @@
           <t>https://www.linkedin.com/search/results/companies/?keywords=Distribuidora+del+Caribe+%28demo%29</t>
         </is>
       </c>
-      <c r="Q4" s="11" t="inlineStr">
+      <c r="Q4" s="3" t="inlineStr"/>
+      <c r="R4" s="11" t="inlineStr">
         <is>
           <t>Gerente de Transformación Digital; Talent Acquisition</t>
         </is>
       </c>
-      <c r="R4" s="11" t="inlineStr">
+      <c r="S4" s="11" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/search/results/people/?keywords=Gerente+de+Transformaci%C3%B3n+Digital+Distribuidora+del+Caribe+%28demo%29
 https://www.linkedin.com/search/results/people/?keywords=Talent+Acquisition+Distribuidora+del+Caribe+%28demo%29</t>
         </is>
       </c>
-      <c r="S4" s="3" t="inlineStr">
+      <c r="T4" s="3" t="inlineStr">
         <is>
           <t>hay vacantes</t>
         </is>
       </c>
-      <c r="T4" s="3" t="n">
+      <c r="U4" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="U4" s="3" t="inlineStr"/>
       <c r="V4" s="3" t="inlineStr"/>
       <c r="W4" s="3" t="inlineStr"/>
-      <c r="X4" s="11" t="inlineStr">
+      <c r="X4" s="3" t="inlineStr"/>
+      <c r="Y4" s="11" t="inlineStr">
         <is>
           <t>data/documentos/1-distribuidora-del-caribe-demo/mensaje.md</t>
         </is>
       </c>
-      <c r="Y4" s="11" t="inlineStr">
+      <c r="Z4" s="11" t="inlineStr">
         <is>
           <t>data/documentos/1-distribuidora-del-caribe-demo/carta.md</t>
         </is>
       </c>
-      <c r="Z4" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
+      <c r="AA4" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -1326,45 +1335,46 @@
           <t>https://www.linkedin.com/search/results/companies/?keywords=Servicios+Globales+RD+%28demo%29</t>
         </is>
       </c>
-      <c r="Q5" s="11" t="inlineStr">
+      <c r="Q5" s="3" t="inlineStr"/>
+      <c r="R5" s="11" t="inlineStr">
         <is>
           <t>Talent Acquisition; Gerente de Automatización</t>
         </is>
       </c>
-      <c r="R5" s="11" t="inlineStr">
+      <c r="S5" s="11" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/search/results/people/?keywords=Talent+Acquisition+Servicios+Globales+RD+%28demo%29
 https://www.linkedin.com/search/results/people/?keywords=Gerente+de+Automatizaci%C3%B3n+Servicios+Globales+RD+%28demo%29</t>
         </is>
       </c>
-      <c r="S5" s="3" t="inlineStr">
+      <c r="T5" s="3" t="inlineStr">
         <is>
           <t>no hay</t>
         </is>
       </c>
-      <c r="T5" s="3" t="n">
+      <c r="U5" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="U5" s="3" t="inlineStr"/>
       <c r="V5" s="3" t="inlineStr"/>
-      <c r="W5" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="X5" s="11" t="inlineStr">
+      <c r="W5" s="3" t="inlineStr"/>
+      <c r="X5" s="3" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="Y5" s="11" t="inlineStr">
         <is>
           <t>data/documentos/2-servicios-globales-rd-demo/mensaje.md</t>
         </is>
       </c>
-      <c r="Y5" s="11" t="inlineStr">
+      <c r="Z5" s="11" t="inlineStr">
         <is>
           <t>data/documentos/2-servicios-globales-rd-demo/carta.md</t>
         </is>
       </c>
-      <c r="Z5" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
+      <c r="AA5" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -1452,44 +1462,45 @@
           <t>https://www.linkedin.com/search/results/companies/?keywords=LogiPuerto+RD+%28demo%29</t>
         </is>
       </c>
-      <c r="Q6" s="3" t="inlineStr">
+      <c r="Q6" s="3" t="inlineStr"/>
+      <c r="R6" s="3" t="inlineStr">
         <is>
           <t>Gerente de Operaciones</t>
         </is>
       </c>
-      <c r="R6" s="12" t="inlineStr">
+      <c r="S6" s="12" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/search/results/people/?keywords=Gerente+de+Operaciones+LogiPuerto+RD+%28demo%29</t>
         </is>
       </c>
-      <c r="S6" s="3" t="inlineStr">
+      <c r="T6" s="3" t="inlineStr">
         <is>
           <t>no hay</t>
         </is>
       </c>
-      <c r="T6" s="3" t="n">
+      <c r="U6" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="U6" s="3" t="inlineStr"/>
       <c r="V6" s="3" t="inlineStr"/>
-      <c r="W6" s="3" t="inlineStr">
+      <c r="W6" s="3" t="inlineStr"/>
+      <c r="X6" s="3" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="Y6" s="11" t="inlineStr">
+        <is>
+          <t>data/documentos/5-logipuerto-rd-demo/mensaje.md</t>
+        </is>
+      </c>
+      <c r="Z6" s="11" t="inlineStr">
+        <is>
+          <t>data/documentos/5-logipuerto-rd-demo/carta.md</t>
+        </is>
+      </c>
+      <c r="AA6" s="3" t="inlineStr">
         <is>
           <t>2026-10-28</t>
-        </is>
-      </c>
-      <c r="X6" s="11" t="inlineStr">
-        <is>
-          <t>data/documentos/5-logipuerto-rd-demo/mensaje.md</t>
-        </is>
-      </c>
-      <c r="Y6" s="11" t="inlineStr">
-        <is>
-          <t>data/documentos/5-logipuerto-rd-demo/carta.md</t>
-        </is>
-      </c>
-      <c r="Z6" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1578,49 +1589,50 @@
           <t>https://www.linkedin.com/search/results/companies/?keywords=Telecom+Antillas+%28demo%29</t>
         </is>
       </c>
-      <c r="Q7" s="3" t="inlineStr">
+      <c r="Q7" s="3" t="inlineStr"/>
+      <c r="R7" s="3" t="inlineStr">
         <is>
           <t>Gerente de Canales Digitales</t>
         </is>
       </c>
-      <c r="R7" s="12" t="inlineStr">
+      <c r="S7" s="12" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/search/results/people/?keywords=Gerente+de+Canales+Digitales+Telecom+Antillas+%28demo%29</t>
         </is>
       </c>
-      <c r="S7" s="3" t="inlineStr">
+      <c r="T7" s="3" t="inlineStr">
         <is>
           <t>hay vacantes</t>
         </is>
       </c>
-      <c r="T7" s="3" t="n">
+      <c r="U7" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="U7" s="3" t="inlineStr"/>
       <c r="V7" s="3" t="inlineStr"/>
-      <c r="W7" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="X7" s="11" t="inlineStr">
+      <c r="W7" s="3" t="inlineStr"/>
+      <c r="X7" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="Y7" s="11" t="inlineStr">
         <is>
           <t>data/documentos/4-telecom-antillas-demo/mensaje.md</t>
         </is>
       </c>
-      <c r="Y7" s="11" t="inlineStr">
+      <c r="Z7" s="11" t="inlineStr">
         <is>
           <t>data/documentos/4-telecom-antillas-demo/carta.md</t>
         </is>
       </c>
-      <c r="Z7" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
+      <c r="AA7" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z7"/>
+  <autoFilter ref="A1:AA7"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -1632,7 +1644,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P3" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S3" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId14"/>
@@ -1648,13 +1660,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S6" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S7" r:id="rId33"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1764,7 +1776,7 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -1805,7 +1817,7 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -1846,7 +1858,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -1907,7 +1919,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:48:32</t>
+          <t>2026-10-28 14:52:57</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -1930,7 +1942,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:48:32</t>
+          <t>2026-10-28 14:52:57</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -1953,7 +1965,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:48:32</t>
+          <t>2026-10-28 14:52:57</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -1976,7 +1988,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:48:32</t>
+          <t>2026-10-28 14:52:57</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -1999,7 +2011,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:48:32</t>
+          <t>2026-10-28 14:52:57</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -2022,7 +2034,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:48:32</t>
+          <t>2026-10-28 14:52:57</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -2045,7 +2057,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:48:32</t>
+          <t>2026-10-28 14:52:57</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -2068,7 +2080,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:48:32</t>
+          <t>2026-10-28 14:52:57</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -2091,7 +2103,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:48:32</t>
+          <t>2026-10-28 14:52:57</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -2114,7 +2126,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:48:32</t>
+          <t>2026-10-28 14:52:57</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -2137,7 +2149,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:48:32</t>
+          <t>2026-10-28 14:52:57</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -2160,7 +2172,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:48:32</t>
+          <t>2026-10-28 14:52:57</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -2183,7 +2195,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:48:32</t>
+          <t>2026-10-28 14:52:57</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -2206,7 +2218,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:48:32</t>
+          <t>2026-10-28 14:52:57</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -2229,7 +2241,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:48:32</t>
+          <t>2026-10-28 14:52:57</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -2252,7 +2264,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21 10:48:32</t>
+          <t>2026-10-28 14:52:57</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">

</xml_diff>